<commit_message>
Stage 8 fixes: E-011
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Stability/LM5/WA-2026-027/Results/Interim/LM5_FIRST_PULL_REVIEW_DRAFT_Rev01.xlsx
+++ b/output/archive/WestravelleData/Stability/LM5/WA-2026-027/Results/Interim/LM5_FIRST_PULL_REVIEW_DRAFT_Rev01.xlsx
@@ -89,10 +89,10 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -184,7 +184,7 @@
   <commentList>
     <comment ref="H4" authorId="0" shapeId="0">
       <text>
-        <t>Table still has only the first pull. Check the 6-month row is in before this goes to Lomervessa.</t>
+        <t>Months 0, 1, 3 and 6 are reported for every displayed chamber condition. System suitability is complete for accepted analytical runs; interim review and validation sign-off remain pending.</t>
       </text>
     </comment>
   </commentList>
@@ -198,7 +198,7 @@
     <author>Leon Wu</author>
   </authors>
   <commentList>
-    <comment ref="D6" authorId="0" shapeId="0">
+    <comment ref="E6" authorId="0" shapeId="0">
       <text>
         <t>Pull logged 24/08/2026. Chamber log for this window still to be attached.</t>
       </text>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -512,218 +512,238 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WA/2026/027 LM5 first pull review: INTERIM DRAFT</t>
+          <t>Westravelle Analytical Ltd, a Tarnovell company</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>WA/2026/027 LM5 review through month 6: INTERIM DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Status: interim. Partial results only; conclusions pending later pulls and sign-off.</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>WA/2026/027</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>LIMS</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>WST-26-000862</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Lomervessa Pharma</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Lead</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Alice Penrose</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Sequence owner</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Leon Wu</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Method validation</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Saira Mahmood</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Quote accepted</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>20/01/2026</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Protocol start</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>23/02/2026</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>First pull analysed</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Pulls through month 6 analysed</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>24/08/2026</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Completion</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>To be confirmed</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Result (interim)</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Initial assay (% label claim)</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B19" s="4" t="n">
         <v>99.90000000000001</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Last timepoint reported (months)</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B20" s="4" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Interim observation</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Complies at the pulls reported so far; no OOS results</t>
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Leon Wu</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Interim draft 24/08/2026</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>System suitability</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Complete: accepted sequence set for the displayed pulls under WST-26-000862, LM-5 sequence sheets. Reference injections, blank/carryover and chromatographic suitability checked against the method; reviewed by Saira Mahmood. Interim review remains pending.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -750,14 +770,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ICH chamber programme: pulls reported to date (interim)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Assay as % label claim, impurities as % area. Water by Karl Fischer, % w/w. Later timepoints not yet tested and not shown.</t>
         </is>
@@ -807,21 +827,21 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>0.06</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
@@ -832,28 +852,28 @@
       <c r="G5" s="7" t="n">
         <v>2.2</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>0.06</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
@@ -864,28 +884,28 @@
       <c r="G6" s="7" t="n">
         <v>1.7</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>99.09999999999999</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="3" t="n">
         <v>0.08</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>0.05</v>
       </c>
       <c r="F7" s="7" t="n">
@@ -894,28 +914,28 @@
       <c r="G7" s="7" t="n">
         <v>2.4</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>6</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>99.40000000000001</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F8" s="7" t="n">
@@ -924,28 +944,28 @@
       <c r="G8" s="7" t="n">
         <v>2.2</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="3" t="n">
         <v>0.06</v>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
@@ -956,28 +976,28 @@
       <c r="G9" s="7" t="n">
         <v>2.2</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>99.40000000000001</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="3" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
@@ -988,28 +1008,28 @@
       <c r="G10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>3</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>99.5</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="3" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F11" s="7" t="n">
@@ -1018,28 +1038,28 @@
       <c r="G11" s="7" t="n">
         <v>2.1</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>6</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>99.40000000000001</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="3" t="n">
         <v>0.13</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="3" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F12" s="7" t="n">
@@ -1048,28 +1068,28 @@
       <c r="G12" s="7" t="n">
         <v>2.4</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="3" t="n">
         <v>0.06</v>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
@@ -1080,28 +1100,28 @@
       <c r="G13" s="7" t="n">
         <v>2.2</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>99.5</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="3" t="n">
         <v>0.11</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="3" t="n">
         <v>0.06</v>
       </c>
       <c r="F14" s="7" t="n">
@@ -1110,28 +1130,28 @@
       <c r="G14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="3" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>98.8</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="3" t="n">
         <v>0.19</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="3" t="n">
         <v>0.11</v>
       </c>
       <c r="F15" s="7" t="n">
@@ -1140,37 +1160,37 @@
       <c r="G15" s="7" t="n">
         <v>1.1</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="3" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="3" t="n">
         <v>0.36</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>0.21</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="3" t="n">
         <v>0.68</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
@@ -1200,7 +1220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1211,17 +1231,18 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Pull schedule tracker (partly complete)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>P = pulled and tested, S = scheduled, blank = not yet planned for this row.</t>
         </is>
@@ -1229,168 +1250,202 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Photostability</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Retained samples</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1404,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1421,102 +1476,124 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>First pull analysed</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Pulls through month 6 analysed</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Leon Wu</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>24/08/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Interim review of first pull</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Interim review through month 6</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Alice Penrose</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
+      <c r="D4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Validation of interim results</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Saira Mahmood</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n"/>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Final conclusions</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Alice Penrose</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n"/>
+      <c r="D6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>System suitability: accepted LM-5 pull sequence set under WST-26-000862</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Saira Mahmood</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Complete; analytical runs accepted</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>